<commit_message>
June 26 2025 changes 1
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0042958_VerifyCapitalMarketViewsOnOpportunityCounterpartyPage.xlsx
+++ b/TestData/LV_TMTT0042958_VerifyCapitalMarketViewsOnOpportunityCounterpartyPage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48FD7D7-ECF6-43CC-8471-910DB52DB5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4696A49-B36D-4A0C-81F6-EB9C5F2C61FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -191,12 +191,6 @@
     <t>Comment</t>
   </si>
   <si>
-    <t>CM Stages - Shortened View</t>
-  </si>
-  <si>
-    <t>CM Stages - Extended View</t>
-  </si>
-  <si>
     <t>All</t>
   </si>
   <si>
@@ -257,13 +251,19 @@
     <t>Debt Financing</t>
   </si>
   <si>
-    <t>Lenkrad</t>
-  </si>
-  <si>
     <t>Avanti</t>
   </si>
   <si>
     <t>Equity Placements</t>
+  </si>
+  <si>
+    <t>CS Stages - Extended View</t>
+  </si>
+  <si>
+    <t>CS Stages - Shortened View</t>
+  </si>
+  <si>
+    <t>Project Lenkrad</t>
   </si>
 </sst>
 </file>
@@ -753,13 +753,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -767,7 +767,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -783,20 +783,20 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{850E31EB-B584-4A83-ACBB-1314D996B82C}">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>17</v>
       </c>
@@ -804,7 +804,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -812,7 +812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>19</v>
       </c>
@@ -820,7 +820,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>20</v>
       </c>
@@ -828,7 +828,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
@@ -836,7 +836,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>22</v>
       </c>
@@ -844,7 +844,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>23</v>
       </c>
@@ -852,7 +852,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>24</v>
       </c>
@@ -860,7 +860,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>25</v>
       </c>
@@ -868,7 +868,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>26</v>
       </c>
@@ -876,7 +876,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>27</v>
       </c>
@@ -884,7 +884,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>28</v>
       </c>
@@ -892,61 +892,61 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
       <c r="B15" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
       <c r="B19" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
       <c r="B20" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
       <c r="B21" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
       <c r="B22" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7"/>
       <c r="B23" s="10" t="s">
         <v>47</v>
@@ -960,17 +960,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -983,17 +983,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1007,14 +1007,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D30953EE-CA2E-4F7C-B9BA-21629FCB862C}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1025,12 +1025,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
         <v>14</v>
@@ -1039,15 +1039,15 @@
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
@@ -1056,7 +1056,7 @@
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1068,44 +1068,44 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20D7FA6C-AE2A-4BFF-9BF9-DF691CB2C529}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="C2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>57</v>
-      </c>
-      <c r="B3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1116,33 +1116,33 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1398F625-8674-4D63-93D8-B47E3A580505}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="B4" s="3"/>
     </row>
@@ -1155,34 +1155,34 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD3FF30-5810-42A4-B6D3-B7BD65EBF170}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
     </row>
-    <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
     </row>
   </sheetData>
@@ -1193,83 +1193,83 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C4377B4-D948-4640-A265-48AD96959963}">
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>47</v>
       </c>
@@ -1282,132 +1282,132 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA60E9-1496-427F-875C-4561E659EAD1}">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
ExpenseRequest changes July 17 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0042958_VerifyCapitalMarketViewsOnOpportunityCounterpartyPage.xlsx
+++ b/TestData/LV_TMTT0042958_VerifyCapitalMarketViewsOnOpportunityCounterpartyPage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4696A49-B36D-4A0C-81F6-EB9C5F2C61FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2EFED11-2D4D-46C4-B0B5-1A1F49C3D5C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="72">
   <si>
     <t>James Craven</t>
   </si>
@@ -261,9 +261,6 @@
   </si>
   <si>
     <t>CS Stages - Shortened View</t>
-  </si>
-  <si>
-    <t>Project Lenkrad</t>
   </si>
 </sst>
 </file>
@@ -456,7 +453,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -472,6 +469,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -753,13 +751,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -767,7 +765,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -783,12 +781,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{850E31EB-B584-4A83-ACBB-1314D996B82C}">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>64</v>
       </c>
@@ -796,7 +794,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>17</v>
       </c>
@@ -804,7 +802,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -812,7 +810,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>19</v>
       </c>
@@ -820,7 +818,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>20</v>
       </c>
@@ -828,7 +826,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
@@ -836,7 +834,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>22</v>
       </c>
@@ -844,7 +842,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>23</v>
       </c>
@@ -852,7 +850,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>24</v>
       </c>
@@ -860,7 +858,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>25</v>
       </c>
@@ -868,7 +866,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>26</v>
       </c>
@@ -876,7 +874,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>27</v>
       </c>
@@ -884,7 +882,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>28</v>
       </c>
@@ -892,61 +890,61 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="8"/>
       <c r="B14" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="7"/>
       <c r="B15" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="7"/>
       <c r="B16" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
       <c r="B17" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="7"/>
       <c r="B18" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
       <c r="B19" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="7"/>
       <c r="B20" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="7"/>
       <c r="B21" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
       <c r="B22" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="7"/>
       <c r="B23" s="10" t="s">
         <v>47</v>
@@ -960,17 +958,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -983,17 +981,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1007,14 +1005,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D30953EE-CA2E-4F7C-B9BA-21629FCB862C}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1025,9 +1023,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>72</v>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="s">
+        <v>15</v>
       </c>
       <c r="B2" t="s">
         <v>67</v>
@@ -1035,14 +1033,11 @@
       <c r="C2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="G2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -1068,14 +1063,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20D7FA6C-AE2A-4BFF-9BF9-DF691CB2C529}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>49</v>
       </c>
@@ -1086,7 +1081,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -1097,7 +1092,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>55</v>
       </c>
@@ -1116,31 +1111,31 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1398F625-8674-4D63-93D8-B47E3A580505}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>48</v>
       </c>
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>70</v>
       </c>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -1155,34 +1150,34 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD3FF30-5810-42A4-B6D3-B7BD65EBF170}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
     </row>
-    <row r="7" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6"/>
     </row>
   </sheetData>
@@ -1193,83 +1188,83 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C4377B4-D948-4640-A265-48AD96959963}">
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>47</v>
       </c>
@@ -1282,132 +1277,132 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA60E9-1496-427F-875C-4561E659EAD1}">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>47</v>
       </c>

</xml_diff>